<commit_message>
Hoàn thiện và đồng bộ bộ tài liệu báo cáo dự án
Cập nhật các tài liệu đề xuất, kế hoạch dự án, user story, product backlog, kiến trúc, thiết kế giao diện và cơ sở dữ liệu. Đồng bộ sprint backlog, kế hoạch kiểm thử, test case, test report, biên bản họp, reflection và tài liệu quản lý cấu hình.

Cập nhật bìa tài liệu và báo cáo PDF tổng hợp; chuẩn hóa tên tệp, loại bỏ các bản tài liệu cũ đã được thay thế.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BaoCao_Final/9.2.TestCaseSprint2.xlsx
+++ b/BaoCao_Final/9.2.TestCaseSprint2.xlsx
@@ -3229,7 +3229,7 @@
         <v>17</v>
       </c>
       <c r="H23" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="I23" s="65" t="s">
         <v>63</v>
@@ -3238,7 +3238,7 @@
         <v>17</v>
       </c>
       <c r="K23" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="L23" s="65" t="s">
         <v>63</v>
@@ -3268,7 +3268,7 @@
         <v>17</v>
       </c>
       <c r="H24" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="I24" s="65" t="s">
         <v>63</v>
@@ -3277,7 +3277,7 @@
         <v>17</v>
       </c>
       <c r="K24" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="L24" s="65" t="s">
         <v>63</v>
@@ -3307,7 +3307,7 @@
         <v>17</v>
       </c>
       <c r="H25" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="I25" s="65" t="s">
         <v>63</v>
@@ -3316,7 +3316,7 @@
         <v>17</v>
       </c>
       <c r="K25" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="L25" s="65" t="s">
         <v>63</v>
@@ -3363,7 +3363,7 @@
         <v>17</v>
       </c>
       <c r="H27" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="I27" s="65" t="s">
         <v>63</v>
@@ -3372,7 +3372,7 @@
         <v>17</v>
       </c>
       <c r="K27" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="L27" s="65" t="s">
         <v>63</v>
@@ -3402,7 +3402,7 @@
         <v>17</v>
       </c>
       <c r="H28" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="I28" s="65" t="s">
         <v>52</v>
@@ -3411,7 +3411,7 @@
         <v>17</v>
       </c>
       <c r="K28" s="67">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="L28" s="65" t="s">
         <v>52</v>
@@ -3688,7 +3688,7 @@
         <v>17</v>
       </c>
       <c r="H35" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I35" s="65" t="s">
         <v>63</v>
@@ -3697,7 +3697,7 @@
         <v>17</v>
       </c>
       <c r="K35" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L35" s="65" t="s">
         <v>63</v>
@@ -3725,7 +3725,7 @@
         <v>17</v>
       </c>
       <c r="H36" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I36" s="65" t="s">
         <v>63</v>
@@ -3734,7 +3734,7 @@
         <v>17</v>
       </c>
       <c r="K36" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L36" s="65" t="s">
         <v>63</v>
@@ -3762,7 +3762,7 @@
         <v>17</v>
       </c>
       <c r="H37" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I37" s="65" t="s">
         <v>63</v>
@@ -3771,7 +3771,7 @@
         <v>17</v>
       </c>
       <c r="K37" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L37" s="65" t="s">
         <v>63</v>
@@ -3799,7 +3799,7 @@
         <v>17</v>
       </c>
       <c r="H38" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I38" s="65" t="s">
         <v>63</v>
@@ -3808,7 +3808,7 @@
         <v>17</v>
       </c>
       <c r="K38" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L38" s="65" t="s">
         <v>63</v>
@@ -3836,7 +3836,7 @@
         <v>17</v>
       </c>
       <c r="H39" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I39" s="65" t="s">
         <v>63</v>
@@ -3845,7 +3845,7 @@
         <v>17</v>
       </c>
       <c r="K39" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L39" s="65" t="s">
         <v>63</v>
@@ -3873,7 +3873,7 @@
         <v>17</v>
       </c>
       <c r="H40" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I40" s="65" t="s">
         <v>52</v>
@@ -3882,7 +3882,7 @@
         <v>17</v>
       </c>
       <c r="K40" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L40" s="65" t="s">
         <v>52</v>
@@ -3910,7 +3910,7 @@
         <v>80</v>
       </c>
       <c r="H41" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I41" s="65" t="s">
         <v>52</v>
@@ -3919,7 +3919,7 @@
         <v>17</v>
       </c>
       <c r="K41" s="67">
-        <v>46283</v>
+        <v>46269</v>
       </c>
       <c r="L41" s="65" t="s">
         <v>52</v>
@@ -3969,7 +3969,7 @@
         <v>17</v>
       </c>
       <c r="H43" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I43" s="65" t="s">
         <v>63</v>
@@ -3978,7 +3978,7 @@
         <v>17</v>
       </c>
       <c r="K43" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L43" s="65" t="s">
         <v>63</v>
@@ -4008,7 +4008,7 @@
         <v>17</v>
       </c>
       <c r="H44" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I44" s="65" t="s">
         <v>52</v>
@@ -4017,7 +4017,7 @@
         <v>17</v>
       </c>
       <c r="K44" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L44" s="65" t="s">
         <v>52</v>
@@ -4047,7 +4047,7 @@
         <v>17</v>
       </c>
       <c r="H45" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I45" s="65" t="s">
         <v>52</v>
@@ -4056,7 +4056,7 @@
         <v>17</v>
       </c>
       <c r="K45" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L45" s="65" t="s">
         <v>52</v>
@@ -4086,7 +4086,7 @@
         <v>17</v>
       </c>
       <c r="H46" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="I46" s="65" t="s">
         <v>63</v>
@@ -4095,7 +4095,7 @@
         <v>17</v>
       </c>
       <c r="K46" s="67">
-        <v>46282</v>
+        <v>46268</v>
       </c>
       <c r="L46" s="65" t="s">
         <v>63</v>
@@ -4615,7 +4615,7 @@
         <v>17</v>
       </c>
       <c r="H35" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I35" s="47" t="s">
         <v>114</v>
@@ -4624,7 +4624,7 @@
         <v>17</v>
       </c>
       <c r="K35" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L35" s="47" t="s">
         <v>114</v>
@@ -4652,7 +4652,7 @@
         <v>17</v>
       </c>
       <c r="H36" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I36" s="47" t="s">
         <v>114</v>
@@ -4661,7 +4661,7 @@
         <v>17</v>
       </c>
       <c r="K36" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L36" s="47" t="s">
         <v>114</v>
@@ -4689,7 +4689,7 @@
         <v>17</v>
       </c>
       <c r="H37" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I37" s="47" t="s">
         <v>63</v>
@@ -4698,7 +4698,7 @@
         <v>17</v>
       </c>
       <c r="K37" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L37" s="47" t="s">
         <v>63</v>
@@ -4726,7 +4726,7 @@
         <v>17</v>
       </c>
       <c r="H38" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I38" s="47" t="s">
         <v>63</v>
@@ -4735,7 +4735,7 @@
         <v>17</v>
       </c>
       <c r="K38" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L38" s="47" t="s">
         <v>63</v>
@@ -4763,7 +4763,7 @@
         <v>17</v>
       </c>
       <c r="H39" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I39" s="47" t="s">
         <v>114</v>
@@ -4772,7 +4772,7 @@
         <v>17</v>
       </c>
       <c r="K39" s="48">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L39" s="47" t="s">
         <v>114</v>
@@ -4820,7 +4820,7 @@
         <v>17</v>
       </c>
       <c r="H41" s="53">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I41" s="52" t="s">
         <v>63</v>
@@ -4829,7 +4829,7 @@
         <v>17</v>
       </c>
       <c r="K41" s="53">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L41" s="52" t="s">
         <v>63</v>
@@ -4859,7 +4859,7 @@
         <v>80</v>
       </c>
       <c r="H42" s="53">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I42" s="52" t="s">
         <v>114</v>
@@ -4868,7 +4868,7 @@
         <v>17</v>
       </c>
       <c r="K42" s="53">
-        <v>46283</v>
+        <v>46271</v>
       </c>
       <c r="L42" s="52" t="s">
         <v>114</v>
@@ -4900,7 +4900,7 @@
         <v>17</v>
       </c>
       <c r="H43" s="53">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I43" s="52" t="s">
         <v>63</v>
@@ -4909,7 +4909,7 @@
         <v>17</v>
       </c>
       <c r="K43" s="53">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L43" s="52" t="s">
         <v>63</v>
@@ -4939,7 +4939,7 @@
         <v>17</v>
       </c>
       <c r="H44" s="55">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="I44" s="54" t="s">
         <v>114</v>
@@ -4948,7 +4948,7 @@
         <v>17</v>
       </c>
       <c r="K44" s="55">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="L44" s="54" t="s">
         <v>114</v>
@@ -5549,7 +5549,7 @@
         <v>17</v>
       </c>
       <c r="H35" s="35">
-        <v>46283</v>
+        <v>46277</v>
       </c>
       <c r="I35" s="36" t="s">
         <v>52</v>
@@ -5558,7 +5558,7 @@
         <v>17</v>
       </c>
       <c r="K35" s="35">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="L35" s="36" t="s">
         <v>52</v>
@@ -5605,7 +5605,7 @@
         <v>17</v>
       </c>
       <c r="H37" s="35">
-        <v>46283</v>
+        <v>46277</v>
       </c>
       <c r="I37" s="36" t="s">
         <v>114</v>
@@ -5614,7 +5614,7 @@
         <v>17</v>
       </c>
       <c r="K37" s="35">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="L37" s="36" t="s">
         <v>114</v>
@@ -5644,7 +5644,7 @@
         <v>17</v>
       </c>
       <c r="H38" s="35">
-        <v>46283</v>
+        <v>46277</v>
       </c>
       <c r="I38" s="36" t="s">
         <v>63</v>
@@ -5653,7 +5653,7 @@
         <v>17</v>
       </c>
       <c r="K38" s="35">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="L38" s="36" t="s">
         <v>63</v>
@@ -5917,7 +5917,7 @@
         <v>17</v>
       </c>
       <c r="H35" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="I35" s="36" t="s">
         <v>63</v>
@@ -5926,7 +5926,7 @@
         <v>17</v>
       </c>
       <c r="K35" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="L35" s="36" t="s">
         <v>63</v>
@@ -5956,7 +5956,7 @@
         <v>17</v>
       </c>
       <c r="H36" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="I36" s="36" t="s">
         <v>63</v>
@@ -5965,7 +5965,7 @@
         <v>17</v>
       </c>
       <c r="K36" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="L36" s="36" t="s">
         <v>63</v>
@@ -5995,7 +5995,7 @@
         <v>17</v>
       </c>
       <c r="H37" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="I37" s="36" t="s">
         <v>63</v>
@@ -6004,7 +6004,7 @@
         <v>17</v>
       </c>
       <c r="K37" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="L37" s="36" t="s">
         <v>63</v>
@@ -6034,7 +6034,7 @@
         <v>80</v>
       </c>
       <c r="H38" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="I38" s="36" t="s">
         <v>63</v>
@@ -6043,7 +6043,7 @@
         <v>17</v>
       </c>
       <c r="K38" s="35">
-        <v>46283</v>
+        <v>46274</v>
       </c>
       <c r="L38" s="36" t="s">
         <v>63</v>
@@ -6091,7 +6091,7 @@
         <v>17</v>
       </c>
       <c r="H40" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="I40" s="36" t="s">
         <v>52</v>
@@ -6100,7 +6100,7 @@
         <v>17</v>
       </c>
       <c r="K40" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="L40" s="36" t="s">
         <v>52</v>
@@ -6130,7 +6130,7 @@
         <v>17</v>
       </c>
       <c r="H41" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="I41" s="36" t="s">
         <v>52</v>
@@ -6139,7 +6139,7 @@
         <v>17</v>
       </c>
       <c r="K41" s="35">
-        <v>46283</v>
+        <v>46273</v>
       </c>
       <c r="L41" s="36" t="s">
         <v>52</v>
@@ -6169,7 +6169,7 @@
         <v>17</v>
       </c>
       <c r="H42" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="I42" s="36" t="s">
         <v>63</v>
@@ -6178,7 +6178,7 @@
         <v>17</v>
       </c>
       <c r="K42" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="L42" s="36" t="s">
         <v>63</v>
@@ -6208,7 +6208,7 @@
         <v>17</v>
       </c>
       <c r="H43" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="I43" s="36" t="s">
         <v>114</v>
@@ -6217,7 +6217,7 @@
         <v>17</v>
       </c>
       <c r="K43" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="L43" s="36" t="s">
         <v>114</v>
@@ -6247,7 +6247,7 @@
         <v>17</v>
       </c>
       <c r="H44" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="I44" s="36" t="s">
         <v>114</v>
@@ -6256,7 +6256,7 @@
         <v>17</v>
       </c>
       <c r="K44" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="L44" s="36" t="s">
         <v>114</v>
@@ -6286,7 +6286,7 @@
         <v>17</v>
       </c>
       <c r="H45" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="I45" s="36" t="s">
         <v>114</v>
@@ -6295,7 +6295,7 @@
         <v>17</v>
       </c>
       <c r="K45" s="35">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="L45" s="36" t="s">
         <v>114</v>
@@ -6555,7 +6555,7 @@
         <v>17</v>
       </c>
       <c r="H35" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="I35" s="36" t="s">
         <v>63</v>
@@ -6564,7 +6564,7 @@
         <v>17</v>
       </c>
       <c r="K35" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="L35" s="36" t="s">
         <v>63</v>
@@ -6594,7 +6594,7 @@
         <v>17</v>
       </c>
       <c r="H36" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="I36" s="36" t="s">
         <v>63</v>
@@ -6603,7 +6603,7 @@
         <v>17</v>
       </c>
       <c r="K36" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="L36" s="36" t="s">
         <v>63</v>
@@ -6633,7 +6633,7 @@
         <v>17</v>
       </c>
       <c r="H37" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="I37" s="36" t="s">
         <v>52</v>
@@ -6642,7 +6642,7 @@
         <v>17</v>
       </c>
       <c r="K37" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="L37" s="36" t="s">
         <v>52</v>
@@ -6690,7 +6690,7 @@
         <v>17</v>
       </c>
       <c r="H39" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="I39" s="36" t="s">
         <v>52</v>
@@ -6699,7 +6699,7 @@
         <v>17</v>
       </c>
       <c r="K39" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="L39" s="36" t="s">
         <v>52</v>
@@ -6729,7 +6729,7 @@
         <v>17</v>
       </c>
       <c r="H40" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="I40" s="36" t="s">
         <v>114</v>
@@ -6738,7 +6738,7 @@
         <v>17</v>
       </c>
       <c r="K40" s="35">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="L40" s="36" t="s">
         <v>114</v>
@@ -7024,7 +7024,7 @@
         <v>17</v>
       </c>
       <c r="H35" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="I35" s="7" t="s">
         <v>63</v>
@@ -7033,7 +7033,7 @@
         <v>17</v>
       </c>
       <c r="K35" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="L35" s="7" t="s">
         <v>63</v>
@@ -7063,7 +7063,7 @@
         <v>17</v>
       </c>
       <c r="H36" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="I36" s="7" t="s">
         <v>52</v>
@@ -7072,7 +7072,7 @@
         <v>17</v>
       </c>
       <c r="K36" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="L36" s="7" t="s">
         <v>52</v>
@@ -7120,7 +7120,7 @@
         <v>17</v>
       </c>
       <c r="H38" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="I38" s="7" t="s">
         <v>63</v>
@@ -7129,7 +7129,7 @@
         <v>17</v>
       </c>
       <c r="K38" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="L38" s="7" t="s">
         <v>63</v>
@@ -7159,7 +7159,7 @@
         <v>17</v>
       </c>
       <c r="H39" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="I39" s="7" t="s">
         <v>52</v>
@@ -7168,7 +7168,7 @@
         <v>17</v>
       </c>
       <c r="K39" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="L39" s="7" t="s">
         <v>52</v>
@@ -7198,7 +7198,7 @@
         <v>17</v>
       </c>
       <c r="H40" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="I40" s="7" t="s">
         <v>52</v>
@@ -7207,7 +7207,7 @@
         <v>17</v>
       </c>
       <c r="K40" s="6">
-        <v>46283</v>
+        <v>46272</v>
       </c>
       <c r="L40" s="7" t="s">
         <v>52</v>

</xml_diff>